<commit_message>
xlstream-eval: add Excel-recalculated conformance fixture for issue 137
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/issues/issue-137-cross-sheet-simple-aggregate.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/issues/issue-137-cross-sheet-simple-aggregate.xlsx
@@ -1,35 +1,66 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream-issue-137/crates/xlstream-eval/tests/fixtures/issues/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_25F82EEB8BCCDEC708671AD73AD4E217A2D0431F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -48,80 +79,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -409,66 +381,58 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2">
         <v>1000</v>
       </c>
       <c r="B2">
         <f>SUM(Sheet2!A2:A4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3">
         <v>2000</v>
       </c>
       <c r="B3">
         <f>AVERAGE(Sheet2!A2:A4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B4">
         <f>COUNT(Sheet2!A2:A4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B5">
         <f>MAX(Sheet2!A2:A4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B6">
         <f>MIN(Sheet2!A2:A4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B7">
         <f>COUNTA(Sheet2!A:A)</f>
-        <v/>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -477,33 +441,27 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2">
         <v>10</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3">
         <v>20</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4">
         <v>30</v>
       </c>
     </row>

</xml_diff>

<commit_message>
xlstream-eval: consolidate issue-137 tests into conformance fixture
Replace inline integration tests with a single conformance fixture
covering cross-sheet aggregates, mixed main+cross, and multi-sheet
isolation. Also fixes cross-sheet bounded range collection.
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/issues/issue-137-cross-sheet-simple-aggregate.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/issues/issue-137-cross-sheet-simple-aggregate.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream-issue-137/crates/xlstream-eval/tests/fixtures/issues/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_25F82EEB8BCCDEC708671AD73AD4E217A2D0431F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_64E644448142E60AFD0CE5FB5BAB7E54E60232B6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Value</t>
   </si>
@@ -42,7 +43,19 @@
     <t>Result</t>
   </si>
   <si>
+    <t>Mixed</t>
+  </si>
+  <si>
+    <t>MultiSheet</t>
+  </si>
+  <si>
     <t>Data</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Y</t>
   </si>
 </sst>
 </file>
@@ -382,18 +395,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1000</v>
       </c>
@@ -401,8 +420,16 @@
         <f>SUM(Sheet2!A2:A4)</f>
         <v>60</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C2">
+        <f>SUM(A2:A3)</f>
+        <v>3000</v>
+      </c>
+      <c r="D2">
+        <f>SUM(Sheet2!A2:A4)</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2000</v>
       </c>
@@ -410,26 +437,34 @@
         <f>AVERAGE(Sheet2!A2:A4)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C3">
+        <f>SUM(Sheet2!A2:A4)</f>
+        <v>60</v>
+      </c>
+      <c r="D3">
+        <f>MAX(Sheet3!B2:B4)</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B4">
         <f>COUNT(Sheet2!A2:A4)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B5">
         <f>MAX(Sheet2!A2:A4)</f>
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B6">
         <f>MIN(Sheet2!A2:A4)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B7">
         <f>COUNTA(Sheet2!A:A)</f>
         <v>4</v>
@@ -447,7 +482,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
@@ -463,6 +498,39 @@
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B4">
+        <v>300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>